<commit_message>
feat(masterdata): DodgeStage 표 + 서든데스·하한 설정
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#DodgeConfig.xlsx
+++ b/table/Datas/#DodgeConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,6 +522,26 @@
           <t>tile_on_seconds</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>min_interval_seconds</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>min_warn_seconds</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sudden_death_base</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>sudden_death_growth</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -629,6 +649,26 @@
           <t>float</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -741,6 +781,26 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>tile_on_seconds</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>min_interval_seconds</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>min_warn_seconds</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>sudden_death_base</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>sudden_death_growth</t>
         </is>
       </c>
     </row>
@@ -804,6 +864,18 @@
       </c>
       <c r="U5" t="n">
         <v>0.55</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="X5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>